<commit_message>
Day 19 task 1 to 4 JSON
</commit_message>
<xml_diff>
--- a/playwright/tests/testData/TestData.xlsx
+++ b/playwright/tests/testData/TestData.xlsx
@@ -209,11 +209,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="d-m-yy"/>
-    <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,6 +224,12 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -247,7 +252,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -286,6 +291,13 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFff0000"/>
       </left>
@@ -324,41 +336,41 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -393,7 +405,7 @@
       <totalsRowFormula>Sum</totalsRowFormula>
     </tableColumn>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium9" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
 </table>
 </file>
 
@@ -740,7 +752,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="41.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -778,7 +790,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="41.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="40.5" customFormat="1" s="1">
       <c r="A3" s="8" t="s">
         <v>24</v>
       </c>
@@ -816,7 +828,7 @@
         <v>33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="41.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="44.25" customFormat="1" s="1">
       <c r="A4" s="11" t="s">
         <v>24</v>
       </c>
@@ -854,7 +866,7 @@
         <v>41</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="44.25" customFormat="1" s="1">
       <c r="A5" s="11" t="s">
         <v>24</v>
       </c>
@@ -892,7 +904,7 @@
         <v>50</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
@@ -906,7 +918,7 @@
       <c r="K6" s="11"/>
       <c r="L6" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A7" s="11"/>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -920,7 +932,7 @@
       <c r="K7" s="11"/>
       <c r="L7" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -934,7 +946,7 @@
       <c r="K8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A9" s="11"/>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
@@ -948,7 +960,7 @@
       <c r="K9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="20.05" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A10" s="11"/>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
@@ -962,7 +974,7 @@
       <c r="K10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="20.05" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A11" s="11"/>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
@@ -976,7 +988,7 @@
       <c r="K11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="20.05" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -1130,7 +1142,7 @@
       <c r="K22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A23" s="11"/>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>

</xml_diff>